<commit_message>
aula dia 18/02/2026, trabalhando com Excel no Python
</commit_message>
<xml_diff>
--- a/aula199/workbook.xlsx
+++ b/aula199/workbook.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C3" t="n">
         <v>9.699999999999999</v>
@@ -483,6 +483,84 @@
       </c>
       <c r="C5" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rondi</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>35</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>João</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9.699999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Luiz</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rondi</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>35</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
aula dia 19/02/2026 trabalhando com excel e imagens (pillow)
</commit_message>
<xml_diff>
--- a/aula199/workbook.xlsx
+++ b/aula199/workbook.xlsx
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C3" t="n">
         <v>9.699999999999999</v>
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C8" t="n">
         <v>9.699999999999999</v>

</xml_diff>